<commit_message>
feat: add mockup for academic results dashboard with charts and tables
- Implemented a new component `ResultadosDashboard` for displaying academic results.
- Added example data for students, questions, and evolution metrics.
- Integrated various charts using Recharts for visual representation of data.
- Created tables for displaying student performance and question metrics.
- Enhanced UI with KPIs and interactive elements for better user experience.
- Introduced temporal configuration handling in `NewIndicatorDrawer` for managing sorting levels.
</commit_message>
<xml_diff>
--- a/data/database/indicators.xlsx
+++ b/data/database/indicators.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,6 +464,11 @@
           <t>filter_dimensions</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>temporal_config</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -482,7 +487,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-12 23:56:35</t>
+          <t>2026-03-13 00:18:30</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -493,6 +498,11 @@
       <c r="G2" t="inlineStr">
         <is>
           <t>[4, 5, 8, 9]</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>{"levels": [{"label": "Año", "sort_mode": "numeric", "order": []}, {"label": "Mes", "sort_mode": "custom", "order": []}]}</t>
         </is>
       </c>
     </row>
@@ -513,17 +523,22 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-12 23:56:57</t>
+          <t>2026-03-13 00:21:53</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>{"logro_1": [{"metric_id": 6, "column": "Logro"}, {"metric_id": 7, "column": "Logro"}], "nivel_de_logro": [{"metric_id": 6, "column": "Nivel Logro"}, {"metric_id": 7, "column": "Nivel Logro"}], "habilidad": [{"metric_id": 6, "column": "Habilidad"}, {"metric_id": 7, "column": "Habilidad"}], "habilidad_2": [{"metric_id": 7, "column": "Eje Temático"}], "evaluacion_num": [{"metric_id": 6, "column": "Hito"}, {"metric_id": 7, "column": "Hito"}]}</t>
+          <t>{"logro_1": [{"metric_id": 6, "column": "Logro"}, {"metric_id": 7, "column": "Logro"}], "nivel_de_logro": [{"metric_id": 6, "column": "Nivel Logro"}, {"metric_id": 7, "column": "Nivel Logro"}], "habilidad": [{"metric_id": 6, "column": "Habilidad"}, {"metric_id": 7, "column": "Habilidad"}], "habilidad_2": [{"metric_id": 7, "column": "Eje Temático"}], "evaluacion_num": [{"metric_id": 6, "column": "Hito"}, {"metric_id": 7, "column": "Hito"}], "logro_2": [{"metric_id": 6, "column": "Logro Promedio"}]}</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>[3, 5, 4, 8]</t>
+          <t>[3, 5, 4, 8, 14]</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>{}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor charts and data processing to support dynamic formatting and temporal labels
- Updated various chart components to utilize new formatting functions for values and domains.
- Introduced roleFormats prop to handle different formatting requirements across charts.
- Enhanced data processing to build temporal labels based on configuration, allowing for better representation of evaluation numbers.
- Modified the dashboard renderer to pass down new props for role formats and temporal configurations.
- Improved error handling and data validation in the Results page for fetching initial data.
</commit_message>
<xml_diff>
--- a/data/database/indicators.xlsx
+++ b/data/database/indicators.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -479,6 +479,16 @@
           <t>achievement_levels</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>dashboard_layout</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>role_formats</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -497,12 +507,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-13 19:43:56</t>
+          <t>2026-03-17 08:19:07</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>{"logro_1": [{"metric_id": 4, "column": "Rend"}, {"metric_id": 5, "column": "Logro"}], "logro_2": [{"metric_id": 4, "column": "SIMCE"}], "nivel_de_logro": [{"metric_id": 4, "column": "Logro"}, {"metric_id": 5, "column": "Logro"}], "habilidad": [{"metric_id": 5, "column": "Habilidad"}], "habilidad_2": [{"metric_id": 5, "column": "Eje Temático"}], "evaluacion_num": [{"metric_id": 4, "column": "Mes"}, {"metric_id": 5, "column": "Mes"}, {"metric_id": 4, "column": "Año"}, {"metric_id": 5, "column": "Año"}]}</t>
+          <t>{"logro_1": [{"metric_id": 4, "column": "Rend"}, {"metric_id": 5, "column": "Logro"}], "logro_2": [{"metric_id": 4, "column": "SIMCE"}], "nivel_de_logro": [{"metric_id": 4, "column": "Logro"}, {"metric_id": 5, "column": "Logro"}], "habilidad": [{"metric_id": 5, "column": "Habilidad"}, {"metric_id": 5, "column": "Eje Temático"}], "habilidad_2": [{"metric_id": 5, "column": "Eje Temático"}], "evaluacion_num": [{"metric_id": 4, "column": "Mes"}, {"metric_id": 5, "column": "Mes"}, {"metric_id": 4, "column": "Año"}, {"metric_id": 5, "column": "Año"}]}</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -523,6 +533,16 @@
       <c r="J2" t="inlineStr">
         <is>
           <t>["Insuficiente", "Elemental", "Adecuado"]</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>{"tabs": [{"id": "general", "label": "Vista General", "rows": [{"cols": 4, "items": [{"type": "kpis"}]}, {"cols": 1, "items": [{"type": "table", "component": "TablaResumenCursos"}]}, {"cols": 2, "items": [{"type": "chart", "component": "GraficoLogroPorCurso", "requires": ["logro_1"]}, {"type": "chart", "component": "GraficoBoxplotPorCurso", "requires": ["logro_1"]}]}, {"cols": 2, "items": [{"type": "chart", "component": "GraficoDistribucionNiveles", "requires": ["nivel_de_logro"]}, {"type": "chart", "component": "GraficoNivelesPorCurso", "requires": ["nivel_de_logro"]}]}]}, {"id": "curso", "label": "Detalle Curso", "rows": [{"cols": 1, "items": [{"type": "course_selector"}]}, {"cols": 2, "items": [{"type": "chart", "component": "GraficoHabilidades", "requires": ["habilidad"], "dimension": "habilidad"}, {"type": "chart", "component": "GraficoHabilidades", "requires": ["habilidad_2"], "dimension": "habilidad_2"}]}, {"cols": 1, "items": [{"type": "table", "component": "TablaAlumnos"}]}, {"cols": 1, "items": [{"type": "table", "component": "TablaPreguntas"}]}]}, {"id": "tab_1773742631382", "label": "Tendencia", "rows": [{"cols": 2, "items": [{"type": "chart", "component": "GraficoTendenciaTemporal", "requires": ["logro_1", "evaluacion_num"]}, {"type": "chart", "component": "GraficoPromedioAgrupadoPorDimension", "requires": ["logro_1", "evaluacion_num"]}]}, {"cols": 2, "items": [{"type": "chart", "component": "GraficoNivelesPorCursoYMes", "requires": ["nivel_de_logro", "evaluacion_num"]}]}]}]}</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>{"logro_2": "#.0"}</t>
         </is>
       </c>
     </row>
@@ -543,7 +563,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-13 19:44:08</t>
+          <t>2026-03-17 08:19:24</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -553,7 +573,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>[3, 5, 4, 8, 14]</t>
+          <t>[3, 4, 8, 14, 15]</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -569,6 +589,16 @@
       <c r="J3" t="inlineStr">
         <is>
           <t>["Inicial", "Intermedio", "Avanzado"]</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>{"tabs": [{"id": "general", "label": "Vista General", "rows": [{"cols": 4, "items": [{"type": "kpis"}]}, {"cols": 1, "items": [{"type": "table", "component": "TablaResumenCursos"}]}, {"cols": 2, "items": [{"type": "chart", "component": "GraficoLogroPorCurso", "requires": ["logro_1"]}, {"type": "chart", "component": "GraficoBoxplotPorCurso", "requires": ["logro_1"]}]}, {"cols": 2, "items": [{"type": "chart", "component": "GraficoDistribucionNiveles", "requires": ["nivel_de_logro"]}, {"type": "chart", "component": "GraficoNivelesPorCurso", "requires": ["nivel_de_logro"]}]}]}, {"id": "curso", "label": "Detalle Curso", "rows": [{"cols": 1, "items": [{"type": "course_selector"}]}, {"cols": 2, "items": [{"type": "chart", "component": "GraficoHabilidades", "requires": ["habilidad"]}, {"type": "chart", "component": "GraficoHabilidades", "requires": ["habilidad_2"], "dimension": "habilidad_2"}]}, {"cols": 1, "items": [{"type": "table", "component": "TablaAlumnos"}]}, {"cols": 1, "items": [{"type": "table", "component": "TablaPreguntas"}]}]}, {"id": "tab_1773744775707", "label": "Tendencia", "rows": [{"cols": 2, "items": [{"type": "chart", "component": "GraficoTendenciaTemporal", "requires": ["logro_1", "evaluacion_num"]}, {"type": "chart", "component": "GraficoPromedioAgrupadoPorDimension", "requires": ["logro_1", "evaluacion_num"]}]}, {"cols": 1, "items": [{"type": "chart", "component": "GraficoNivelesPorCursoYMes", "requires": ["nivel_de_logro", "evaluacion_num"]}]}]}]}</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>{}</t>
         </is>
       </c>
     </row>
@@ -589,12 +619,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-03-17 00:22:36</t>
+          <t>2026-03-17 08:36:08</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>{"logro_1": [{"metric_id": 8, "column": "Puntaje"}], "nivel_de_logro": [{"metric_id": 8, "column": "Nivel de Riesgo"}], "evaluacion_num": [{"metric_id": 8, "column": "Versión"}, {"metric_id": 8, "column": "Año"}]}</t>
+          <t>{"logro_1": [{"metric_id": 8, "column": "Puntaje"}], "nivel_de_logro": [{"metric_id": 8, "column": "Nivel de Riesgo"}], "evaluacion_num": [{"metric_id": 8, "column": "Versión"}, {"metric_id": 8, "column": "Año"}], "habilidad": [{"metric_id": 8, "column": "Evaluación"}]}</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -615,6 +645,16 @@
       <c r="J4" t="inlineStr">
         <is>
           <t>["Crítico", "Alto Riesgo", "Cierto Riesgo", "Bajo Riesgo"]</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>{"tabs": [{"id": "general", "label": "Vista General", "rows": [{"cols": 4, "items": [{"type": "kpis"}]}, {"cols": 1, "items": [{"type": "table", "component": "TablaResumenCursos"}]}, {"cols": 2, "items": [{"type": "chart", "component": "GraficoLogroPorCurso", "requires": ["logro_1"]}, {"type": "chart", "component": "GraficoBoxplotPorCurso", "requires": ["logro_1"]}]}, {"cols": 2, "items": [{"type": "chart", "component": "GraficoDistribucionNiveles", "requires": ["nivel_de_logro"]}, {"type": "chart", "component": "GraficoNivelesPorCurso", "requires": ["nivel_de_logro"]}]}]}, {"id": "curso", "label": "Detalle Curso", "rows": [{"cols": 1, "items": [{"type": "course_selector"}]}, {"cols": 1, "items": [{"type": "chart", "component": "GraficoHabilidades", "requires": ["habilidad"]}]}, {"cols": 1, "items": [{"type": "table", "component": "TablaAlumnos"}]}, {"cols": 1, "items": [{"type": "table", "component": "TablaPreguntas"}]}]}, {"id": "tab_1773745127342", "label": "Habilidades", "rows": [{"cols": 1, "items": [{"type": "course_selector"}]}, {"cols": 1, "items": [{"type": "chart", "component": "GraficoRadarHabilidades", "requires": ["habilidad"], "dimension": "habilidad"}]}]}]}</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>{"logro_1": "#.0"}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add DoubleGroupedBar chart and enhance existing chart components
- Introduced DoubleGroupedBar component for double grouping visualization.
- Updated GroupedBarByPeriod to alias DoubleGroupedBar for backward compatibility.
- Enhanced various chart components (BarByGroup, HorizontalBarByDimension, BoxPlotByGroup, etc.) to accept additional props for labels and legend visibility.
- Refactored data processing to normalize field names and maintain backward compatibility with legacy role aliases.
- Improved layout and margin handling in charts to accommodate new label props.
- Added support for conditional display of values in charts.
</commit_message>
<xml_diff>
--- a/data/database/indicators.xlsx
+++ b/data/database/indicators.xlsx
@@ -507,7 +507,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-21 00:01:49</t>
+          <t>2026-03-21 14:45:06</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -537,7 +537,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>{"tabs": [{"id": "general", "label": "Vista General", "rows": [{"cols": 4, "items": [{"type": "kpis"}]}, {"cols": 1, "items": [{"type": "table", "component": "TablaResumenCursos"}]}, {"cols": 2, "items": [{"type": "chart", "component": "BarByGroup", "valueField": ["_rend", "_simce"], "groupField": "_curso"}, {"type": "chart", "component": "BoxPlotByGroup", "valueField": ["_rend", "_simce"], "groupField": "_curso"}]}, {"cols": 2, "items": [{"type": "chart", "component": "PieComposition", "categoryField": "_logro"}, {"type": "chart", "component": "StackedCountByGroup", "groupField": "_curso", "categoryField": "_logro"}]}]}, {"id": "curso", "label": "Detalle Curso", "rows": [{"cols": 1, "items": [{"type": "course_selector"}]}, {"cols": 2, "items": [{"type": "chart", "component": "HorizontalBarByDimension", "dimensionField": "_habilidad", "valueField": "_rend"}, {"type": "chart", "component": "HorizontalBarByDimension", "dimensionField": "_habilidad_2", "valueField": "_rend"}]}, {"cols": 1, "items": [{"type": "table", "component": "TablaAlumnos"}]}, {"cols": 1, "items": [{"type": "table", "component": "TablaPreguntas"}]}]}, {"id": "tab_1773742631382", "label": "Tendencia", "rows": [{"cols": 2, "items": [{"type": "chart", "component": "TrendLine", "groupField": "_curso", "periodField": "_evaluacion_num", "valueField": ["_rend", "_simce"]}, {"type": "chart", "component": "GraficoPromedioAgrupadoPorDimension", "requires": ["logro_1", "evaluacion_num"]}, {"type": "chart", "component": "GroupedBarByPeriod", "groupField": "_curso", "periodField": "_evaluacion_num", "valueField": ["_rend", "_simce"]}]}, {"cols": 2, "items": [{"type": "chart", "component": "GraficoNivelesPorCursoYMes", "requires": ["nivel_de_logro", "evaluacion_num"]}]}, {"cols": 1, "items": [{"type": "chart", "component": "StackedCountByGroup", "groupField": "_curso", "categoryField": "_logro"}, {"type": "chart", "component": "StackedCountByGroupAndPeriod", "groupField": "_curso", "periodField": "_evaluacion_num", "categoryField": "_logro"}]}]}]}</t>
+          <t>{"tabs": [{"id": "general", "label": "Vista General", "rows": [{"cols": 4, "items": [{"type": "kpis"}]}, {"cols": 1, "items": [{"type": "table", "component": "TablaResumenCursos"}]}, {"cols": 2, "items": [{"type": "chart", "component": "BarByGroup", "valueField": ["_rend", "_simce"], "groupField": "_curso"}, {"type": "chart", "component": "BoxPlotByGroup", "valueField": ["_rend", "_simce"], "groupField": "_curso"}]}, {"cols": 2, "items": [{"type": "chart", "component": "PieComposition", "categoryField": "_logro"}, {"type": "chart", "component": "StackedCountByGroup", "groupField": "_curso", "categoryField": "_logro"}]}]}, {"id": "curso", "label": "Detalle Curso", "rows": [{"cols": 1, "items": [{"type": "course_selector"}]}, {"cols": 2, "items": [{"type": "chart", "component": "HorizontalBarByDimension", "dimensionField": "_habilidad", "valueField": "_rend"}, {"type": "chart", "component": "HorizontalBarByDimension", "dimensionField": "_habilidad_2", "valueField": "_rend"}]}, {"cols": 1, "items": [{"type": "table", "component": "TablaAlumnos"}]}, {"cols": 1, "items": [{"type": "table", "component": "TablaPreguntas"}]}]}, {"id": "tab_1773742631382", "label": "Tendencia", "rows": [{"cols": 2, "items": [{"type": "chart", "component": "DoubleGroupedBar", "groupField": "_curso", "subGroupField": "_mes", "valueField": "_rend", "showValues": true, "title": "Avance entre pruebas por curso"}]}, {"cols": 2, "items": [{"type": "chart", "component": "GraficoNivelesPorCursoYMes", "requires": ["nivel_de_logro", "evaluacion_num"]}]}, {"cols": 1, "items": [{"type": "chart", "component": "StackedCountByGroup", "groupField": "_curso", "categoryField": "_logro"}, {"type": "chart", "component": "StackedCountByGroupAndPeriod", "groupField": "_curso", "periodField": "_evaluacion_num", "categoryField": "_logro"}]}]}, {"id": "tab_1774109207699", "label": "Prueba", "rows": [{"cols": 2, "items": [{"type": "chart", "component": "BoxPlotByGroup", "valueField": "_rend", "groupField": "_curso"}, {"type": "chart", "component": "PieComposition", "categoryField": "_logro", "showLegend": true, "title": "Composición por Nivel"}, {"type": "chart", "component": "PieComposition", "categoryField": "_logro", "title": "Este es un título de prueba", "showLegend": false}]}, {"cols": 1, "items": []}]}]}</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">

</xml_diff>